<commit_message>
Partite: orari ritrovo/inizio, fix avversario su tablet, import aggiorna invece di duplicare
</commit_message>
<xml_diff>
--- a/public/templates/calendario-partite-template.xlsx
+++ b/public/templates/calendario-partite-template.xlsx
@@ -418,15 +418,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -452,12 +454,22 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Ora ritrovo</t>
+          <t>Ora ritrovo andata</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Ora inizio</t>
+          <t>Ora inizio andata</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Ora ritrovo ritorno</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Ora inizio ritorno</t>
         </is>
       </c>
     </row>
@@ -492,6 +504,16 @@
           <t>15:00</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -516,12 +538,22 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>15:30</t>
         </is>
       </c>
     </row>
@@ -554,6 +586,16 @@
       <c r="F4" t="inlineStr">
         <is>
           <t>15:30</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>15:00</t>
         </is>
       </c>
     </row>
@@ -573,10 +615,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="100" customWidth="1" min="1" max="1"/>
+    <col width="105" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -596,7 +638,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2. Data andata: la data della partita del girone di andata (gg/mm/aaaa).</t>
+          <t>2. Data andata: data della partita del girone di andata (gg/mm/aaaa).</t>
         </is>
       </c>
     </row>
@@ -617,56 +659,70 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>5. Data ritorno: la data della partita del girone di ritorno (gg/mm/aaaa).</t>
+          <t>5. Data ritorno: data della partita del girone di ritorno (gg/mm/aaaa).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6. Ora ritrovo / Ora inizio (facoltative): formato HH:MM, es. 14:00. Valgono sia per andata che per ritorno.</t>
+          <t>ORARI (facoltativi, formato HH:MM, es. 14:00) — SEPARATI per andata e ritorno:</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Il programma crea automaticamente:</t>
+          <t>6. Ora ritrovo andata / Ora inizio andata: orari della partita di ANDATA.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>- la partita di andata con i dati inseriti;</t>
+          <t>7. Ora ritrovo ritorno / Ora inizio ritorno: orari della partita di RITORNO.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>- la partita di ritorno, stessa avversaria, ma con casa/trasferta invertita rispetto all'andata.</t>
+          <t>Il programma crea automaticamente:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Se ricarichi il file dopo aver corretto qualcosa, le partite gia' presenti in quelle date vengono AGGIORNATE, non duplicate.</t>
+          <t>- la partita di andata con i dati e gli orari di andata;</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Le 3 righe di esempio nel foglio "Calendario" sono solo dimostrative: cancellale e inserisci le tue partite.</t>
+          <t>- la partita di ritorno, stessa avversaria, casa/trasferta invertita rispetto all'andata, con gli orari di ritorno.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Dopo aver compilato, salva il file e caricalo nella sezione Ricorrenze &gt; Partite &gt; Metodo 2, selezionando la categoria corretta.</t>
+          <t>Se ricarichi il file dopo aver corretto qualcosa, le partite gia' presenti in quelle date vengono AGGIORNATE, non duplicate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Le 3 righe di esempio nel foglio "Calendario" sono solo dimostrative: cancellale e inserisci le tue partite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Dopo aver compilato, salva il file e caricalo in Ricorrenze &gt; Partite &gt; Metodo 2, selezionando la categoria.</t>
         </is>
       </c>
     </row>

</xml_diff>